<commit_message>
usability penalty for undefended First improvement to the playing strength in a long time!  Thanks to SynapticResonance for pointing out this strategy. Renamed usability and defendability methods to more general names.
</commit_message>
<xml_diff>
--- a/tests/summary.xlsx
+++ b/tests/summary.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="20225"/>
-  <workbookPr autoCompressPictures="0"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr autoCompressPictures="0" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="17500" yWindow="4280" windowWidth="26220" windowHeight="15920"/>
+    <workbookView xWindow="17505" yWindow="4335" windowWidth="26220" windowHeight="15855"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="140001" concurrentCalc="0"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="55">
   <si>
     <t>file</t>
   </si>
@@ -159,6 +159,33 @@
   </si>
   <si>
     <t>keeping defendable</t>
+  </si>
+  <si>
+    <t>undefended defendable and 1-usable</t>
+  </si>
+  <si>
+    <t>undefended defendable vs undefended defendable and 1-usable.txt</t>
+  </si>
+  <si>
+    <t>undefended defendable vs undefended defendable and 1-usable 2.txt</t>
+  </si>
+  <si>
+    <t>undefended defendable vs undefended defendable and 1-usable 3.txt</t>
+  </si>
+  <si>
+    <t>full</t>
+  </si>
+  <si>
+    <t>undefended defendable vs undefended defendable and 1-usable 4.txt</t>
+  </si>
+  <si>
+    <t>improves the strength for longer words, decreases for shorter words</t>
+  </si>
+  <si>
+    <t>I'm going to use the 1-usable thing in player0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -533,23 +560,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+  <dimension ref="A1:N29"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.140625" customWidth="1"/>
+    <col min="9" max="9" width="4.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="47" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="66.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="65.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="66.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -593,7 +620,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>20</v>
       </c>
@@ -638,7 +665,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>20</v>
       </c>
@@ -683,7 +710,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>20</v>
       </c>
@@ -725,7 +752,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>20</v>
       </c>
@@ -767,7 +794,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E6" s="2"/>
       <c r="F6" s="1">
         <f>SUM(F2:F5)</f>
@@ -782,10 +809,10 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>20</v>
       </c>
@@ -830,7 +857,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>20</v>
       </c>
@@ -875,7 +902,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>20</v>
       </c>
@@ -917,7 +944,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>20</v>
       </c>
@@ -959,7 +986,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F12" s="1">
         <f>SUM(F8:F11)</f>
         <v>94</v>
@@ -973,7 +1000,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>20</v>
       </c>
@@ -1018,7 +1045,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>20</v>
       </c>
@@ -1063,7 +1090,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>20</v>
       </c>
@@ -1108,7 +1135,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>20</v>
       </c>
@@ -1153,7 +1180,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F18" s="1">
         <f>SUM(F14:F17)</f>
         <v>88</v>
@@ -1167,11 +1194,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>20</v>
       </c>
@@ -1216,7 +1243,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1236,7 +1263,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -1256,7 +1283,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>20</v>
       </c>
@@ -1271,6 +1298,190 @@
       </c>
       <c r="E23">
         <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>60</v>
+      </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" t="s">
+        <v>42</v>
+      </c>
+      <c r="E26">
+        <v>8</v>
+      </c>
+      <c r="F26">
+        <v>76</v>
+      </c>
+      <c r="G26">
+        <v>63.5</v>
+      </c>
+      <c r="H26">
+        <f>F26-G26</f>
+        <v>12.5</v>
+      </c>
+      <c r="I26">
+        <v>53</v>
+      </c>
+      <c r="J26">
+        <v>14</v>
+      </c>
+      <c r="K26">
+        <v>6</v>
+      </c>
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="M26" t="s">
+        <v>49</v>
+      </c>
+      <c r="N26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>60</v>
+      </c>
+      <c r="B27" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27">
+        <v>12</v>
+      </c>
+      <c r="F27">
+        <v>66</v>
+      </c>
+      <c r="G27">
+        <v>66.5</v>
+      </c>
+      <c r="H27">
+        <f>F27-G27</f>
+        <v>-0.5</v>
+      </c>
+      <c r="I27">
+        <v>54</v>
+      </c>
+      <c r="J27">
+        <v>29</v>
+      </c>
+      <c r="K27">
+        <v>3</v>
+      </c>
+      <c r="L27">
+        <v>3</v>
+      </c>
+      <c r="M27" t="s">
+        <v>48</v>
+      </c>
+      <c r="N27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>60</v>
+      </c>
+      <c r="B28" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28">
+        <v>25</v>
+      </c>
+      <c r="F28">
+        <f>21+20+22.5</f>
+        <v>63.5</v>
+      </c>
+      <c r="G28">
+        <f>23+26+23.5</f>
+        <v>72.5</v>
+      </c>
+      <c r="H28">
+        <f>F28-G28</f>
+        <v>-9</v>
+      </c>
+      <c r="I28">
+        <f>18+17+19</f>
+        <v>54</v>
+      </c>
+      <c r="J28">
+        <f>10+5+7</f>
+        <v>22</v>
+      </c>
+      <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28">
+        <v>5</v>
+      </c>
+      <c r="M28" t="s">
+        <v>47</v>
+      </c>
+      <c r="N28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" t="s">
+        <v>50</v>
+      </c>
+      <c r="E29">
+        <v>25</v>
+      </c>
+      <c r="F29">
+        <v>27.5</v>
+      </c>
+      <c r="G29">
+        <v>36</v>
+      </c>
+      <c r="H29">
+        <f>F29-G29</f>
+        <v>-8.5</v>
+      </c>
+      <c r="I29">
+        <v>26</v>
+      </c>
+      <c r="J29">
+        <v>19</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>4</v>
+      </c>
+      <c r="M29" t="s">
+        <v>51</v>
+      </c>
+      <c r="N29" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1287,7 +1498,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -1301,7 +1512,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>

</xml_diff>